<commit_message>
updates to plotting files
</commit_message>
<xml_diff>
--- a/TunnelDataProcessing/BoundaryLayerComparison/BoundaryLayerComparison.xlsx
+++ b/TunnelDataProcessing/BoundaryLayerComparison/BoundaryLayerComparison.xlsx
@@ -18,7 +18,151 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="78">
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
+  <si>
+    <t>Y_over_D</t>
+  </si>
+  <si>
+    <t>Mach</t>
+  </si>
+  <si>
+    <t>Mach_nd</t>
+  </si>
   <si>
     <t>Y_over_D</t>
   </si>
@@ -163,13 +307,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
@@ -1292,20 +1436,20 @@
   <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" customWidth="true"/>
-    <col min="2" max="2" width="12.5546875" customWidth="true"/>
-    <col min="3" max="3" width="12.5546875" customWidth="true"/>
+    <col min="1" max="1" width="13.7109375" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>58</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
@@ -2428,20 +2572,20 @@
   <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" customWidth="true"/>
-    <col min="2" max="2" width="12.5546875" customWidth="true"/>
-    <col min="3" max="3" width="12.5546875" customWidth="true"/>
+    <col min="1" max="1" width="13.7109375" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
@@ -3571,13 +3715,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2">
@@ -6896,13 +7040,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2">

</xml_diff>